<commit_message>
Remove local paths and user name from workbook metadata
Strip the saved workbook path, the cached folder values and the hyperlink display path, and normalize author metadata.
</commit_message>
<xml_diff>
--- a/Реестры.xlsx
+++ b/Реестры.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\valk\projects\payment-registry-automation\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B7729B-55BB-447E-9BD4-737CBF6197FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25420" windowHeight="16300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -1642,7 +1637,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="valk" refreshedDate="46302.510031712962" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="219" xr:uid="{A3786681-B250-4DE7-BA29-A03FFF724B5B}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Валерий Кравченко" refreshedDate="46302.510031712962" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="219" xr:uid="{A3786681-B250-4DE7-BA29-A03FFF724B5B}">
   <cacheSource type="worksheet">
     <worksheetSource name="Реестры"/>
   </cacheSource>
@@ -5064,12 +5059,12 @@
       </c>
       <c r="B2" s="2" t="str" cm="1">
         <f t="array" aca="1" ref="B2" ca="1">LEFT(CELL("filename",A1),FIND("[",CELL("имяфайла",A1))-1)&amp;"data\registries\"</f>
-        <v>\\wsl.localhost\Ubuntu\home\valk\projects\payment-registry-automation\data\registries\</v>
+        <v>C:\Examples\payment-registry-automation\data\registries\</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="\\wsl.localhost\Ubuntu\home\valk\projects\payment-registry-automation\data\registries\" xr:uid="{0702D99C-A98B-4712-BC27-43A262BC8850}"/>
+    <hyperlink ref="B2" r:id="rId1" display="C:\Examples\payment-registry-automation\data\registries\" xr:uid="{0702D99C-A98B-4712-BC27-43A262BC8850}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>